<commit_message>
Some changes from AVD Oct-17-2023
</commit_message>
<xml_diff>
--- a/TestData/T1426_OpportunityToEngagementConversionMappingForCFJobTypes2.xlsx
+++ b/TestData/T1426_OpportunityToEngagementConversionMappingForCFJobTypes2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6A60F8-5658-40EE-A866-962583DCD60D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D63180-E1E8-40FE-BCB3-695CA967DE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="14610" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>

</xml_diff>